<commit_message>
feat(F-NAR-019): TREE-AUT-027 polish Le manteau bleu de Mila au marché
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-027.xlsx
+++ b/stories/arbres/TREE-AUT-027.xlsx
@@ -2753,17 +2753,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle pose un cube, près de la caisse froide. Les carreaux de la cuisine restent dans ses pieds. Un cube attrape un reflet d'orange, au stand.</t>
+          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Je pose un cube, près de la caisse froide. Un froid de carreaux reste sous ses chaussons. Un cube attrape un reflet d'orange, au stand.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle pose un cube, près de la caisse froide. Les carreaux de la cuisine restent dans ses pieds. Un cube attrape un reflet d'orange, au stand.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Je pose un cube, près de la caisse froide. Un froid de carreaux reste sous ses chaussons. Un cube attrape un reflet d'orange, au stand.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle pose un cube, près de la caisse froide. Les carreaux de la cuisine restent dans ses pieds. Un cube attrape un reflet d'orange, au stand. [pause]</t>
+          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Je pose un cube, près de la caisse froide. Un froid de carreaux reste sous ses chaussons. Un cube attrape un reflet d'orange, au stand. [pause]</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -2910,8 +2910,8 @@
 narrateur|Elle soulève le pan, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, toute ronde.
-narrateur|Elle pose un cube, près de la caisse froide.
-narrateur|Les carreaux de la cuisine restent dans ses pieds.
+enfant-f|Je pose un cube, près de la caisse froide.
+narrateur|Un froid de carreaux reste sous ses chaussons.
 narrateur|Un cube attrape un reflet d'orange, au stand.</t>
         </is>
       </c>
@@ -3132,17 +3132,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle pose un cube, près de la chaise tiède. L'odeur de menthe de l'évier la suit. Un cube attrape un reflet d'orange, au stand.</t>
+          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Je pose un cube, près de la chaise tiède. L'odeur de menthe de l'évier la suit. Un cube attrape un reflet d'orange, au stand.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle pose un cube, près de la chaise tiède. L'odeur de menthe de l'évier la suit. Un cube attrape un reflet d'orange, au stand.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Je pose un cube, près de la chaise tiède. L'odeur de menthe de l'évier la suit. Un cube attrape un reflet d'orange, au stand.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle pose un cube, près de la chaise tiède. L'odeur de menthe de l'évier la suit. Un cube attrape un reflet d'orange, au stand. [pause]</t>
+          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Je pose un cube, près de la chaise tiède. L'odeur de menthe de l'évier la suit. Un cube attrape un reflet d'orange, au stand. [pause]</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -3289,7 +3289,7 @@
 narrateur|Elle soulève le col, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, un peu chaude.
-narrateur|Elle pose un cube, près de la chaise tiède.
+enfant-f|Je pose un cube, près de la chaise tiède.
 narrateur|L'odeur de menthe de l'évier la suit.
 narrateur|Un cube attrape un reflet d'orange, au stand.</t>
         </is>
@@ -3511,17 +3511,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle pose un cube, près de la caisse des lampes. Le col ouvert de la cuisine tient chaud. Un cube attrape un reflet d'orange, au stand.</t>
+          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Je pose un cube, près de la caisse des lampes. Le col ouvert lui tient chaud, dehors. Un cube attrape un reflet d'orange, au stand.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle pose un cube, près de la caisse des lampes. Le col ouvert de la cuisine tient chaud. Un cube attrape un reflet d'orange, au stand.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Je pose un cube, près de la caisse des lampes. Le col ouvert lui tient chaud, dehors. Un cube attrape un reflet d'orange, au stand.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle pose un cube, près de la caisse des lampes. Le col ouvert de la cuisine tient chaud. Un cube attrape un reflet d'orange, au stand. [pause]</t>
+          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Je pose un cube, près de la caisse des lampes. Le col ouvert lui tient chaud, dehors. Un cube attrape un reflet d'orange, au stand. [pause]</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -3668,8 +3668,8 @@
 narrateur|Elle soulève le pli, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, parfumée.
-narrateur|Elle pose un cube, près de la caisse des lampes.
-narrateur|Le col ouvert de la cuisine tient chaud.
+enfant-f|Je pose un cube, près de la caisse des lampes.
+narrateur|Le col ouvert lui tient chaud, dehors.
 narrateur|Un cube attrape un reflet d'orange, au stand.</t>
         </is>
       </c>
@@ -4285,17 +4285,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle ouvre le livre, près des oranges froides. Les carreaux de la cuisine restent dans ses pieds. Une miette d'orange reste au bord de la page.</t>
+          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. J'ouvre le livre, près des oranges froides. Un froid de carreaux reste sous ses chaussons. Une miette d'orange reste au bord de la page.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle ouvre le livre, près des oranges froides. Les carreaux de la cuisine restent dans ses pieds. Une miette d'orange reste au bord de la page.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. J'ouvre le livre, près des oranges froides. Un froid de carreaux reste sous ses chaussons. Une miette d'orange reste au bord de la page.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle ouvre le livre, près des oranges froides. Les carreaux de la cuisine restent dans ses pieds. Une miette d'orange reste au bord de la page. [pause]</t>
+          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. J'ouvre le livre, près des oranges froides. Un froid de carreaux reste sous ses chaussons. Une miette d'orange reste au bord de la page. [pause]</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -4442,8 +4442,8 @@
 narrateur|Elle soulève le pan, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, toute ronde.
-narrateur|Elle ouvre le livre, près des oranges froides.
-narrateur|Les carreaux de la cuisine restent dans ses pieds.
+enfant-f|J'ouvre le livre, près des oranges froides.
+narrateur|Un froid de carreaux reste sous ses chaussons.
 narrateur|Une miette d'orange reste au bord de la page.</t>
         </is>
       </c>
@@ -4664,17 +4664,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle ouvre le livre, près des oranges tièdes. L'odeur de menthe de l'évier la suit. Une miette d'orange reste au bord de la page.</t>
+          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. J'ouvre le livre, près des oranges tièdes. L'odeur de menthe de l'évier la suit. Une miette d'orange reste au bord de la page.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle ouvre le livre, près des oranges tièdes. L'odeur de menthe de l'évier la suit. Une miette d'orange reste au bord de la page.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. J'ouvre le livre, près des oranges tièdes. L'odeur de menthe de l'évier la suit. Une miette d'orange reste au bord de la page.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle ouvre le livre, près des oranges tièdes. L'odeur de menthe de l'évier la suit. Une miette d'orange reste au bord de la page. [pause]</t>
+          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. J'ouvre le livre, près des oranges tièdes. L'odeur de menthe de l'évier la suit. Une miette d'orange reste au bord de la page. [pause]</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4821,7 +4821,7 @@
 narrateur|Elle soulève le col, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, un peu chaude.
-narrateur|Elle ouvre le livre, près des oranges tièdes.
+enfant-f|J'ouvre le livre, près des oranges tièdes.
 narrateur|L'odeur de menthe de l'évier la suit.
 narrateur|Une miette d'orange reste au bord de la page.</t>
         </is>
@@ -5043,17 +5043,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle ouvre le livre, sous les lampes du stand. Le col ouvert de la cuisine tient chaud. Une miette d'orange reste au bord de la page.</t>
+          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. J'ouvre le livre, sous les lampes du stand. Le col ouvert lui tient chaud, dehors. Une miette d'orange reste au bord de la page.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle ouvre le livre, sous les lampes du stand. Le col ouvert de la cuisine tient chaud. Une miette d'orange reste au bord de la page.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. J'ouvre le livre, sous les lampes du stand. Le col ouvert lui tient chaud, dehors. Une miette d'orange reste au bord de la page.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle ouvre le livre, sous les lampes du stand. Le col ouvert de la cuisine tient chaud. Une miette d'orange reste au bord de la page. [pause]</t>
+          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. J'ouvre le livre, sous les lampes du stand. Le col ouvert lui tient chaud, dehors. Une miette d'orange reste au bord de la page. [pause]</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -5200,8 +5200,8 @@
 narrateur|Elle soulève le pli, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, parfumée.
-narrateur|Elle ouvre le livre, sous les lampes du stand.
-narrateur|Le col ouvert de la cuisine tient chaud.
+enfant-f|J'ouvre le livre, sous les lampes du stand.
+narrateur|Le col ouvert lui tient chaud, dehors.
 narrateur|Une miette d'orange reste au bord de la page.</t>
         </is>
       </c>
@@ -5817,17 +5817,17 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle pose une tasse, près de la caisse froide. Les carreaux de la cuisine restent dans ses pieds. La petite casserole est près du vrai bol, dehors.</t>
+          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Je pose une tasse, près de la caisse froide. Un froid de carreaux reste sous ses chaussons. La petite casserole est près du vrai bol, dehors.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle pose une tasse, près de la caisse froide. Les carreaux de la cuisine restent dans ses pieds. La petite casserole est près du vrai bol, dehors.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Je pose une tasse, près de la caisse froide. Un froid de carreaux reste sous ses chaussons. La petite casserole est près du vrai bol, dehors.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle pose une tasse, près de la caisse froide. Les carreaux de la cuisine restent dans ses pieds. La petite casserole est près du vrai bol, dehors. [pause]</t>
+          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Je pose une tasse, près de la caisse froide. Un froid de carreaux reste sous ses chaussons. La petite casserole est près du vrai bol, dehors. [pause]</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -5974,8 +5974,8 @@
 narrateur|Elle soulève le pan, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, toute ronde.
-narrateur|Elle pose une tasse, près de la caisse froide.
-narrateur|Les carreaux de la cuisine restent dans ses pieds.
+enfant-f|Je pose une tasse, près de la caisse froide.
+narrateur|Un froid de carreaux reste sous ses chaussons.
 narrateur|La petite casserole est près du vrai bol, dehors.</t>
         </is>
       </c>
@@ -6196,17 +6196,17 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle pose une tasse, près de la chaise tiède. L'odeur de menthe de l'évier la suit. La petite casserole est près du vrai bol, dehors.</t>
+          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Je pose une tasse, près de la chaise tiède. L'odeur de menthe de l'évier la suit. La petite casserole est près du vrai bol, dehors.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle pose une tasse, près de la chaise tiède. L'odeur de menthe de l'évier la suit. La petite casserole est près du vrai bol, dehors.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Je pose une tasse, près de la chaise tiède. L'odeur de menthe de l'évier la suit. La petite casserole est près du vrai bol, dehors.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle pose une tasse, près de la chaise tiède. L'odeur de menthe de l'évier la suit. La petite casserole est près du vrai bol, dehors. [pause]</t>
+          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Je pose une tasse, près de la chaise tiède. L'odeur de menthe de l'évier la suit. La petite casserole est près du vrai bol, dehors. [pause]</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -6353,7 +6353,7 @@
 narrateur|Elle soulève le col, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, un peu chaude.
-narrateur|Elle pose une tasse, près de la chaise tiède.
+enfant-f|Je pose une tasse, près de la chaise tiède.
 narrateur|L'odeur de menthe de l'évier la suit.
 narrateur|La petite casserole est près du vrai bol, dehors.</t>
         </is>
@@ -6575,17 +6575,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle pose une tasse, sous les lampes du stand. Le col ouvert de la cuisine tient chaud. La petite casserole est près du vrai bol, dehors.</t>
+          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Je pose une tasse, sous les lampes du stand. Le col ouvert lui tient chaud, dehors. La petite casserole est près du vrai bol, dehors.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle pose une tasse, sous les lampes du stand. Le col ouvert de la cuisine tient chaud. La petite casserole est près du vrai bol, dehors.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Je pose une tasse, sous les lampes du stand. Le col ouvert lui tient chaud, dehors. La petite casserole est près du vrai bol, dehors.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle pose une tasse, sous les lampes du stand. Le col ouvert de la cuisine tient chaud. La petite casserole est près du vrai bol, dehors. [pause]</t>
+          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Je pose une tasse, sous les lampes du stand. Le col ouvert lui tient chaud, dehors. La petite casserole est près du vrai bol, dehors. [pause]</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -6732,8 +6732,8 @@
 narrateur|Elle soulève le pli, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, parfumée.
-narrateur|Elle pose une tasse, sous les lampes du stand.
-narrateur|Le col ouvert de la cuisine tient chaud.
+enfant-f|Je pose une tasse, sous les lampes du stand.
+narrateur|Le col ouvert lui tient chaud, dehors.
 narrateur|La petite casserole est près du vrai bol, dehors.</t>
         </is>
       </c>
@@ -8109,17 +8109,17 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle pose un cube, près de la caisse froide. Les bottes font ploc, sur les pavés froids. L'herbe tache un cube, tout vert, au stand.</t>
+          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Je pose un cube, près de la caisse froide. Les bottes font ploc, sur les pavés froids. L'herbe tache un cube, tout vert, au stand.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle pose un cube, près de la caisse froide. Les bottes font ploc, sur les pavés froids. L'herbe tache un cube, tout vert, au stand.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Je pose un cube, près de la caisse froide. Les bottes font ploc, sur les pavés froids. L'herbe tache un cube, tout vert, au stand.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle pose un cube, près de la caisse froide. Les bottes font ploc, sur les pavés froids. L'herbe tache un cube, tout vert, au stand. [pause]</t>
+          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Je pose un cube, près de la caisse froide. Les bottes font ploc, sur les pavés froids. L'herbe tache un cube, tout vert, au stand. [pause]</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -8266,7 +8266,7 @@
 narrateur|Elle soulève le pan, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, toute ronde.
-narrateur|Elle pose un cube, près de la caisse froide.
+enfant-f|Je pose un cube, près de la caisse froide.
 narrateur|Les bottes font ploc, sur les pavés froids.
 narrateur|L'herbe tache un cube, tout vert, au stand.</t>
         </is>
@@ -8488,17 +8488,17 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle pose un cube, près de la chaise tiède. La menthe de la poche sent fort, tout vert. L'herbe tache un cube, tout vert, au stand.</t>
+          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Je pose un cube, près de la chaise tiède. La menthe de la poche sent fort, tout vert. L'herbe tache un cube, tout vert, au stand.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle pose un cube, près de la chaise tiède. La menthe de la poche sent fort, tout vert. L'herbe tache un cube, tout vert, au stand.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Je pose un cube, près de la chaise tiède. La menthe de la poche sent fort, tout vert. L'herbe tache un cube, tout vert, au stand.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle pose un cube, près de la chaise tiède. La menthe de la poche sent fort, tout vert. L'herbe tache un cube, tout vert, au stand. [pause]</t>
+          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Je pose un cube, près de la chaise tiède. La menthe de la poche sent fort, tout vert. L'herbe tache un cube, tout vert, au stand. [pause]</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -8645,7 +8645,7 @@
 narrateur|Elle soulève le col, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, un peu chaude.
-narrateur|Elle pose un cube, près de la chaise tiède.
+enfant-f|Je pose un cube, près de la chaise tiède.
 narrateur|La menthe de la poche sent fort, tout vert.
 narrateur|L'herbe tache un cube, tout vert, au stand.</t>
         </is>
@@ -8867,17 +8867,17 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle pose un cube, près de la caisse des lampes. Une goutte du jardin glisse du manteau bleu. L'herbe tache un cube, tout vert, au stand.</t>
+          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Je pose un cube, près de la caisse des lampes. Une goutte du jardin glisse du manteau bleu. L'herbe tache un cube, tout vert, au stand.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle pose un cube, près de la caisse des lampes. Une goutte du jardin glisse du manteau bleu. L'herbe tache un cube, tout vert, au stand.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Je pose un cube, près de la caisse des lampes. Une goutte du jardin glisse du manteau bleu. L'herbe tache un cube, tout vert, au stand.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle pose un cube, près de la caisse des lampes. Une goutte du jardin glisse du manteau bleu. L'herbe tache un cube, tout vert, au stand. [pause]</t>
+          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Je pose un cube, près de la caisse des lampes. Une goutte du jardin glisse du manteau bleu. L'herbe tache un cube, tout vert, au stand. [pause]</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -9024,7 +9024,7 @@
 narrateur|Elle soulève le pli, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, parfumée.
-narrateur|Elle pose un cube, près de la caisse des lampes.
+enfant-f|Je pose un cube, près de la caisse des lampes.
 narrateur|Une goutte du jardin glisse du manteau bleu.
 narrateur|L'herbe tache un cube, tout vert, au stand.</t>
         </is>
@@ -9641,17 +9641,17 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle ouvre le livre, près des oranges froides. Les bottes font ploc, sur les pavés froids. Une vraie feuille de menthe marque la page.</t>
+          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. J'ouvre le livre, près des oranges froides. Les bottes font ploc, sur les pavés froids. Une vraie feuille de menthe marque la page.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle ouvre le livre, près des oranges froides. Les bottes font ploc, sur les pavés froids. Une vraie feuille de menthe marque la page.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. J'ouvre le livre, près des oranges froides. Les bottes font ploc, sur les pavés froids. Une vraie feuille de menthe marque la page.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle ouvre le livre, près des oranges froides. Les bottes font ploc, sur les pavés froids. Une vraie feuille de menthe marque la page. [pause]</t>
+          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. J'ouvre le livre, près des oranges froides. Les bottes font ploc, sur les pavés froids. Une vraie feuille de menthe marque la page. [pause]</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -9798,7 +9798,7 @@
 narrateur|Elle soulève le pan, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, toute ronde.
-narrateur|Elle ouvre le livre, près des oranges froides.
+enfant-f|J'ouvre le livre, près des oranges froides.
 narrateur|Les bottes font ploc, sur les pavés froids.
 narrateur|Une vraie feuille de menthe marque la page.</t>
         </is>
@@ -10020,17 +10020,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle ouvre le livre, près des oranges tièdes. La menthe de la poche sent fort, tout vert. Une vraie feuille de menthe marque la page.</t>
+          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. J'ouvre le livre, près des oranges tièdes. La menthe de la poche sent fort, tout vert. Une vraie feuille de menthe marque la page.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle ouvre le livre, près des oranges tièdes. La menthe de la poche sent fort, tout vert. Une vraie feuille de menthe marque la page.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. J'ouvre le livre, près des oranges tièdes. La menthe de la poche sent fort, tout vert. Une vraie feuille de menthe marque la page.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle ouvre le livre, près des oranges tièdes. La menthe de la poche sent fort, tout vert. Une vraie feuille de menthe marque la page. [pause]</t>
+          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. J'ouvre le livre, près des oranges tièdes. La menthe de la poche sent fort, tout vert. Une vraie feuille de menthe marque la page. [pause]</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -10177,7 +10177,7 @@
 narrateur|Elle soulève le col, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, un peu chaude.
-narrateur|Elle ouvre le livre, près des oranges tièdes.
+enfant-f|J'ouvre le livre, près des oranges tièdes.
 narrateur|La menthe de la poche sent fort, tout vert.
 narrateur|Une vraie feuille de menthe marque la page.</t>
         </is>
@@ -10399,17 +10399,17 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle ouvre le livre, sous les lampes du stand. Une goutte du jardin glisse du manteau bleu. Une vraie feuille de menthe marque la page.</t>
+          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. J'ouvre le livre, sous les lampes du stand. Une goutte du jardin glisse du manteau bleu. Une vraie feuille de menthe marque la page.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle ouvre le livre, sous les lampes du stand. Une goutte du jardin glisse du manteau bleu. Une vraie feuille de menthe marque la page.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. J'ouvre le livre, sous les lampes du stand. Une goutte du jardin glisse du manteau bleu. Une vraie feuille de menthe marque la page.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle ouvre le livre, sous les lampes du stand. Une goutte du jardin glisse du manteau bleu. Une vraie feuille de menthe marque la page. [pause]</t>
+          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. J'ouvre le livre, sous les lampes du stand. Une goutte du jardin glisse du manteau bleu. Une vraie feuille de menthe marque la page. [pause]</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -10556,7 +10556,7 @@
 narrateur|Elle soulève le pli, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, parfumée.
-narrateur|Elle ouvre le livre, sous les lampes du stand.
+enfant-f|J'ouvre le livre, sous les lampes du stand.
 narrateur|Une goutte du jardin glisse du manteau bleu.
 narrateur|Une vraie feuille de menthe marque la page.</t>
         </is>
@@ -11173,17 +11173,17 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle pose une tasse, près de la caisse froide. Les bottes font ploc, sur les pavés froids. Une goutte perle au bord de l'assiette, dehors.</t>
+          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Je pose une tasse, près de la caisse froide. Les bottes font ploc, sur les pavés froids. Une goutte perle au bord de l'assiette, dehors.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle pose une tasse, près de la caisse froide. Les bottes font ploc, sur les pavés froids. Une goutte perle au bord de l'assiette, dehors.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Je pose une tasse, près de la caisse froide. Les bottes font ploc, sur les pavés froids. Une goutte perle au bord de l'assiette, dehors.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle pose une tasse, près de la caisse froide. Les bottes font ploc, sur les pavés froids. Une goutte perle au bord de l'assiette, dehors. [pause]</t>
+          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Je pose une tasse, près de la caisse froide. Les bottes font ploc, sur les pavés froids. Une goutte perle au bord de l'assiette, dehors. [pause]</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -11330,7 +11330,7 @@
 narrateur|Elle soulève le pan, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, toute ronde.
-narrateur|Elle pose une tasse, près de la caisse froide.
+enfant-f|Je pose une tasse, près de la caisse froide.
 narrateur|Les bottes font ploc, sur les pavés froids.
 narrateur|Une goutte perle au bord de l'assiette, dehors.</t>
         </is>
@@ -11552,17 +11552,17 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle pose une tasse, près de la chaise tiède. La menthe de la poche sent fort, tout vert. Une goutte perle au bord de l'assiette, dehors.</t>
+          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Je pose une tasse, près de la chaise tiède. La menthe de la poche sent fort, tout vert. Une goutte perle au bord de l'assiette, dehors.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle pose une tasse, près de la chaise tiède. La menthe de la poche sent fort, tout vert. Une goutte perle au bord de l'assiette, dehors.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Je pose une tasse, près de la chaise tiède. La menthe de la poche sent fort, tout vert. Une goutte perle au bord de l'assiette, dehors.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle pose une tasse, près de la chaise tiède. La menthe de la poche sent fort, tout vert. Une goutte perle au bord de l'assiette, dehors. [pause]</t>
+          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Je pose une tasse, près de la chaise tiède. La menthe de la poche sent fort, tout vert. Une goutte perle au bord de l'assiette, dehors. [pause]</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -11709,7 +11709,7 @@
 narrateur|Elle soulève le col, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, un peu chaude.
-narrateur|Elle pose une tasse, près de la chaise tiède.
+enfant-f|Je pose une tasse, près de la chaise tiède.
 narrateur|La menthe de la poche sent fort, tout vert.
 narrateur|Une goutte perle au bord de l'assiette, dehors.</t>
         </is>
@@ -11931,17 +11931,17 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle pose une tasse, sous les lampes du stand. Une goutte du jardin glisse du manteau bleu. Une goutte perle au bord de l'assiette, dehors.</t>
+          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Je pose une tasse, sous les lampes du stand. Une goutte du jardin glisse du manteau bleu. Une goutte perle au bord de l'assiette, dehors.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle pose une tasse, sous les lampes du stand. Une goutte du jardin glisse du manteau bleu. Une goutte perle au bord de l'assiette, dehors.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Je pose une tasse, sous les lampes du stand. Une goutte du jardin glisse du manteau bleu. Une goutte perle au bord de l'assiette, dehors.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle pose une tasse, sous les lampes du stand. Une goutte du jardin glisse du manteau bleu. Une goutte perle au bord de l'assiette, dehors. [pause]</t>
+          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Je pose une tasse, sous les lampes du stand. Une goutte du jardin glisse du manteau bleu. Une goutte perle au bord de l'assiette, dehors. [pause]</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -12088,7 +12088,7 @@
 narrateur|Elle soulève le pli, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, parfumée.
-narrateur|Elle pose une tasse, sous les lampes du stand.
+enfant-f|Je pose une tasse, sous les lampes du stand.
 narrateur|Une goutte du jardin glisse du manteau bleu.
 narrateur|Une goutte perle au bord de l'assiette, dehors.</t>
         </is>
@@ -13465,17 +13465,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle pose un cube, près de la caisse froide. Le petit panier jouet tapote la caisse. Un cube tapote le parquet, dans sa mémoire.</t>
+          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Je pose un cube, près de la caisse froide. Le petit panier jouet tapote la caisse. Un cube tapote le parquet, dans sa mémoire.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle pose un cube, près de la caisse froide. Le petit panier jouet tapote la caisse. Un cube tapote le parquet, dans sa mémoire.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Je pose un cube, près de la caisse froide. Le petit panier jouet tapote la caisse. Un cube tapote le parquet, dans sa mémoire.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle pose un cube, près de la caisse froide. Le petit panier jouet tapote la caisse. Un cube tapote le parquet, dans sa mémoire. [pause]</t>
+          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Je pose un cube, près de la caisse froide. Le petit panier jouet tapote la caisse. Un cube tapote le parquet, dans sa mémoire. [pause]</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -13622,7 +13622,7 @@
 narrateur|Elle soulève le pan, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, toute ronde.
-narrateur|Elle pose un cube, près de la caisse froide.
+enfant-f|Je pose un cube, près de la caisse froide.
 narrateur|Le petit panier jouet tapote la caisse.
 narrateur|Un cube tapote le parquet, dans sa mémoire.</t>
         </is>
@@ -13844,17 +13844,17 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle pose un cube, près de la chaise tiède. Le rideau jaune reste derrière, à la maison. Un cube tapote le parquet, dans sa mémoire.</t>
+          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Je pose un cube, près de la chaise tiède. Le rideau jaune reste derrière, à la maison. Un cube tapote le parquet, dans sa mémoire.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle pose un cube, près de la chaise tiède. Le rideau jaune reste derrière, à la maison. Un cube tapote le parquet, dans sa mémoire.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Je pose un cube, près de la chaise tiède. Le rideau jaune reste derrière, à la maison. Un cube tapote le parquet, dans sa mémoire.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle pose un cube, près de la chaise tiède. Le rideau jaune reste derrière, à la maison. Un cube tapote le parquet, dans sa mémoire. [pause]</t>
+          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Je pose un cube, près de la chaise tiède. Le rideau jaune reste derrière, à la maison. Un cube tapote le parquet, dans sa mémoire. [pause]</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -14001,7 +14001,7 @@
 narrateur|Elle soulève le col, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, un peu chaude.
-narrateur|Elle pose un cube, près de la chaise tiède.
+enfant-f|Je pose un cube, près de la chaise tiède.
 narrateur|Le rideau jaune reste derrière, à la maison.
 narrateur|Un cube tapote le parquet, dans sa mémoire.</t>
         </is>
@@ -14223,17 +14223,17 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle pose un cube, près de la caisse des lampes. Le savon de la chambre reste sur le col. Un cube tapote le parquet, dans sa mémoire.</t>
+          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Je pose un cube, près de la caisse des lampes. Le savon de la chambre reste sur le col. Un cube tapote le parquet, dans sa mémoire.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle pose un cube, près de la caisse des lampes. Le savon de la chambre reste sur le col. Un cube tapote le parquet, dans sa mémoire.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Je pose un cube, près de la caisse des lampes. Le savon de la chambre reste sur le col. Un cube tapote le parquet, dans sa mémoire.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle pose un cube, près de la caisse des lampes. Le savon de la chambre reste sur le col. Un cube tapote le parquet, dans sa mémoire. [pause]</t>
+          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Je pose un cube, près de la caisse des lampes. Le savon de la chambre reste sur le col. Un cube tapote le parquet, dans sa mémoire. [pause]</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -14380,7 +14380,7 @@
 narrateur|Elle soulève le pli, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, parfumée.
-narrateur|Elle pose un cube, près de la caisse des lampes.
+enfant-f|Je pose un cube, près de la caisse des lampes.
 narrateur|Le savon de la chambre reste sur le col.
 narrateur|Un cube tapote le parquet, dans sa mémoire.</t>
         </is>
@@ -14997,17 +14997,17 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle ouvre le livre, près des oranges froides. Le petit panier jouet tapote la caisse. Le rideau jaune colore la page, au stand.</t>
+          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. J'ouvre le livre, près des oranges froides. Le petit panier jouet tapote la caisse. Le rideau jaune colore la page, au stand.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle ouvre le livre, près des oranges froides. Le petit panier jouet tapote la caisse. Le rideau jaune colore la page, au stand.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. J'ouvre le livre, près des oranges froides. Le petit panier jouet tapote la caisse. Le rideau jaune colore la page, au stand.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle ouvre le livre, près des oranges froides. Le petit panier jouet tapote la caisse. Le rideau jaune colore la page, au stand. [pause]</t>
+          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. J'ouvre le livre, près des oranges froides. Le petit panier jouet tapote la caisse. Le rideau jaune colore la page, au stand. [pause]</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -15154,7 +15154,7 @@
 narrateur|Elle soulève le pan, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, toute ronde.
-narrateur|Elle ouvre le livre, près des oranges froides.
+enfant-f|J'ouvre le livre, près des oranges froides.
 narrateur|Le petit panier jouet tapote la caisse.
 narrateur|Le rideau jaune colore la page, au stand.</t>
         </is>
@@ -15376,17 +15376,17 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle ouvre le livre, près des oranges tièdes. Le rideau jaune reste derrière, à la maison. Le rideau jaune colore la page, au stand.</t>
+          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. J'ouvre le livre, près des oranges tièdes. Le rideau jaune reste derrière, à la maison. Le rideau jaune colore la page, au stand.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle ouvre le livre, près des oranges tièdes. Le rideau jaune reste derrière, à la maison. Le rideau jaune colore la page, au stand.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. J'ouvre le livre, près des oranges tièdes. Le rideau jaune reste derrière, à la maison. Le rideau jaune colore la page, au stand.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle ouvre le livre, près des oranges tièdes. Le rideau jaune reste derrière, à la maison. Le rideau jaune colore la page, au stand. [pause]</t>
+          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. J'ouvre le livre, près des oranges tièdes. Le rideau jaune reste derrière, à la maison. Le rideau jaune colore la page, au stand. [pause]</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -15533,7 +15533,7 @@
 narrateur|Elle soulève le col, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, un peu chaude.
-narrateur|Elle ouvre le livre, près des oranges tièdes.
+enfant-f|J'ouvre le livre, près des oranges tièdes.
 narrateur|Le rideau jaune reste derrière, à la maison.
 narrateur|Le rideau jaune colore la page, au stand.</t>
         </is>
@@ -15755,17 +15755,17 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle ouvre le livre, sous les lampes du stand. Le savon de la chambre reste sur le col. Le rideau jaune colore la page, au stand.</t>
+          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. J'ouvre le livre, sous les lampes du stand. Le savon de la chambre reste sur le col. Le rideau jaune colore la page, au stand.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle ouvre le livre, sous les lampes du stand. Le savon de la chambre reste sur le col. Le rideau jaune colore la page, au stand.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. J'ouvre le livre, sous les lampes du stand. Le savon de la chambre reste sur le col. Le rideau jaune colore la page, au stand.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle ouvre le livre, sous les lampes du stand. Le savon de la chambre reste sur le col. Le rideau jaune colore la page, au stand. [pause]</t>
+          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. J'ouvre le livre, sous les lampes du stand. Le savon de la chambre reste sur le col. Le rideau jaune colore la page, au stand. [pause]</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -15912,7 +15912,7 @@
 narrateur|Elle soulève le pli, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, parfumée.
-narrateur|Elle ouvre le livre, sous les lampes du stand.
+enfant-f|J'ouvre le livre, sous les lampes du stand.
 narrateur|Le savon de la chambre reste sur le col.
 narrateur|Le rideau jaune colore la page, au stand.</t>
         </is>
@@ -16529,17 +16529,17 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle pose une tasse, près de la caisse froide. Le petit panier jouet tapote la caisse. La petite tasse est près du lit, dans sa poche.</t>
+          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Je pose une tasse, près de la caisse froide. Le petit panier jouet tapote la caisse. La petite tasse est près du lit, dans sa poche.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle pose une tasse, près de la caisse froide. Le petit panier jouet tapote la caisse. La petite tasse est près du lit, dans sa poche.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Je pose une tasse, près de la caisse froide. Le petit panier jouet tapote la caisse. La petite tasse est près du lit, dans sa poche.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Elle pose une tasse, près de la caisse froide. Le petit panier jouet tapote la caisse. La petite tasse est près du lit, dans sa poche. [pause]</t>
+          <t>Le marché s'ouvre, ce matin. Ils sortent, et l'air pique le nez. Mila pose le manteau sur une caisse. J'en prends une, vite ! La bâche se déroule, et recouvre le bleu. Il est sous la bâche, je le vois ! Elle saisit un pan rayé, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous la bâche. L'entaille, je la vois. Elle soulève le pan, sans tirer. Une orange, pour le panier. Mila la choisit, toute ronde. Je pose une tasse, près de la caisse froide. Le petit panier jouet tapote la caisse. La petite tasse est près du lit, dans sa poche. [pause]</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
@@ -16686,7 +16686,7 @@
 narrateur|Elle soulève le pan, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, toute ronde.
-narrateur|Elle pose une tasse, près de la caisse froide.
+enfant-f|Je pose une tasse, près de la caisse froide.
 narrateur|Le petit panier jouet tapote la caisse.
 narrateur|La petite tasse est près du lit, dans sa poche.</t>
         </is>
@@ -16908,17 +16908,17 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle pose une tasse, près de la chaise tiède. Le rideau jaune reste derrière, à la maison. La petite tasse est près du lit, dans sa poche.</t>
+          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Je pose une tasse, près de la chaise tiède. Le rideau jaune reste derrière, à la maison. La petite tasse est près du lit, dans sa poche.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle pose une tasse, près de la chaise tiède. Le rideau jaune reste derrière, à la maison. La petite tasse est près du lit, dans sa poche.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Je pose une tasse, près de la chaise tiède. Le rideau jaune reste derrière, à la maison. La petite tasse est près du lit, dans sa poche.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Elle pose une tasse, près de la chaise tiède. Le rideau jaune reste derrière, à la maison. La petite tasse est près du lit, dans sa poche. [pause]</t>
+          <t>Le marché est plus calme, après la sieste. Ils sortent, et les pavés sont tièdes. Mila pose le manteau sur une chaise. J'en prends une, tiède ! Un sac bleu pend, à côté de la chaise. Il est là, je le vois ! Elle saisit le sac, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, sous le store. L'entaille, je la vois. Elle soulève le col, sans tirer. Une orange, pour le panier. Mila la choisit, un peu chaude. Je pose une tasse, près de la chaise tiède. Le rideau jaune reste derrière, à la maison. La petite tasse est près du lit, dans sa poche. [pause]</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -17065,7 +17065,7 @@
 narrateur|Elle soulève le col, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, un peu chaude.
-narrateur|Elle pose une tasse, près de la chaise tiède.
+enfant-f|Je pose une tasse, près de la chaise tiède.
 narrateur|Le rideau jaune reste derrière, à la maison.
 narrateur|La petite tasse est près du lit, dans sa poche.</t>
         </is>
@@ -17287,17 +17287,17 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle pose une tasse, sous les lampes du stand. Le savon de la chambre reste sur le col. La petite tasse est près du lit, dans sa poche.</t>
+          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le bouton à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Je pose une tasse, sous les lampes du stand. Le savon de la chambre reste sur le col. La petite tasse est près du lit, dans sa poche.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle pose une tasse, sous les lampes du stand. Le savon de la chambre reste sur le col. La petite tasse est près du lit, dans sa poche.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Je pose une tasse, sous les lampes du stand. Le savon de la chambre reste sur le col. La petite tasse est près du lit, dans sa poche.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Elle pose une tasse, sous les lampes du stand. Le savon de la chambre reste sur le col. La petite tasse est près du lit, dans sa poche. [pause]</t>
+          <t>Le marché se range, ce soir. Ils sortent, et la vitre est bleue. Mila pose le manteau près de la caisse. J'en prends une, avant le pli ! La bâche se plie, et avale le bleu. Il est dans le pli, je le vois ! Elle tire le pli, trop vite. Cette fois, elle refuse de foncer. Le &lt;emphasis&gt;bouton&lt;/emphasis&gt; à lune fait toc, dans la bâche. L'entaille, je la vois. Elle soulève le pli, sans tirer. Une orange, pour le panier. Mila la choisit, parfumée. Je pose une tasse, sous les lampes du stand. Le savon de la chambre reste sur le col. La petite tasse est près du lit, dans sa poche. [pause]</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -17444,7 +17444,7 @@
 narrateur|Elle soulève le pli, sans tirer.
 papa|Une orange, pour le panier.
 narrateur|Mila la choisit, parfumée.
-narrateur|Elle pose une tasse, sous les lampes du stand.
+enfant-f|Je pose une tasse, sous les lampes du stand.
 narrateur|Le savon de la chambre reste sur le col.
 narrateur|La petite tasse est près du lit, dans sa poche.</t>
         </is>
@@ -17660,7 +17660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17724,6 +17724,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>